<commit_message>
Update shipment 136782 weights per shipper email
Replace T1-derived per-HS weights with shipper's per-product figures
(DA 144/153, network items 224/255 kg), which reconcile with invoice
and packing list totals (NW 368 / GW 408 kg). T1 discrepancies noted.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CFfffYrcT2goh6WhnHM8g6
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Hitachi_Energy_136782.xlsx
+++ b/output/HS_Code_Summary_Hitachi_Energy_136782.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -670,10 +670,10 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>189.33</v>
+        <v>144</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>238.66</v>
+        <v>153</v>
       </c>
       <c r="E15" s="4" t="n">
         <v>12</v>
@@ -714,10 +714,10 @@
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>178.67</v>
+        <v>224</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>178.67</v>
+        <v>255</v>
       </c>
       <c r="E16" s="4" t="n">
         <v>336</v>
@@ -757,7 +757,7 @@
         <v>368</v>
       </c>
       <c r="D17" s="9" t="n">
-        <v>417.33</v>
+        <v>408</v>
       </c>
       <c r="E17" s="8" t="n">
         <v>348</v>
@@ -802,54 +802,62 @@
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="11" t="inlineStr">
-        <is>
-          <t>• Hmotnosti dle tranzitního dokladu T1 (per položka). Celková hrubá hmotnost dle T1 = 417,33 kg, ale faktura a balicí list uvádějí 408,00 kg — nesoulad 9,33 kg. Čistá hmotnost 368,00 kg souhlasí ve všech dokladech.</t>
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>• Hmotnosti dle e-mailu odesílatele (M. Jahnholz, Hitachi Energy) per produktová řada: Moxa DA 12 ks NW 144 / GW 153 kg; RKS 20 ks NW 104 / GW 115 kg; RM 52 ks NW 10 / GW 15 kg; PT 4 ks NW 6 / GW 10 kg; SFP 260 ks NW 104 / GW 115 kg. Součty (NW 368 / GW 408 kg) souhlasí s fakturou i balicím listem.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>• Množství dle faktury (12 ks serverů). Pozor: T1 deklaruje u HS 847150 celkem 16 ks (pozice 1,2,3,4,13 = 4+4+2+2+4), faktura i balicí list mají 12 ks — pravděpodobně duplicitní pozice v T1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t>• CBAM: nevztahuje se — elektronika/IT zařízení nespadá do působnosti CBAM.</t>
+          <t>• Nesoulad s T1: tranzitní doklad deklaruje hrubou hmotnost celkem 417,33 kg (vs. 408,00 kg) a jiné rozdělení vah na pozice (HS 847150: NW 189,33 kg vs. 144 kg dle odesílatele).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>• Množství dle faktury (12 ks serverů). Pozor: T1 deklaruje u HS 847150 celkem 16 ks (pozice 1,2,3,4,13 = 4+4+2+2+4), faktura, balicí list i e-mail odesílatele mají 12 ks — pravděpodobně duplicitní pozice v T1.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
+          <t>• CBAM: nevztahuje se — elektronika/IT zařízení nespadá do působnosti CBAM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
           <t>• Antidumping: na uvedené HS kódy původu TW nejsou známa antidumpingová cla.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="12" t="inlineStr">
-        <is>
-          <t>• Obchodní sleva: žádná sleva na faktuře — celní hodnoty = fakturované částky (celkem 228 148,00 CHF).</t>
         </is>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="12" t="inlineStr">
         <is>
+          <t>• Obchodní sleva: žádná sleva na faktuře — celní hodnoty = fakturované částky (celkem 228 148,00 CHF).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
           <t>• Doklad T1: zboží se švýcarským statusem T1, celní úřad určení celní úřad Hradec Králové (CZ). Lhůta pro předložení: 17.07.2026.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
     <mergeCell ref="A23:J23"/>
     <mergeCell ref="A22:J22"/>
     <mergeCell ref="A27:J27"/>
     <mergeCell ref="A21:J21"/>
     <mergeCell ref="A28:J28"/>
+    <mergeCell ref="A30:J30"/>
     <mergeCell ref="A29:J29"/>
     <mergeCell ref="A20:J20"/>
     <mergeCell ref="A24:J24"/>

</xml_diff>

<commit_message>
Update shipment 136782 per revised CI/PL rev.1
Gross weight corrected upward to 417.33 kg matching the T1 (pallets
160 + 257 kg per revised packing list). Net weights and quantities
unchanged; corrected T1 still pending verification of the duplicate
server position.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CFfffYrcT2goh6WhnHM8g6
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Hitachi_Energy_136782.xlsx
+++ b/output/HS_Code_Summary_Hitachi_Energy_136782.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -542,328 +542,372 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>870135086 (dated 2026-07-01)</t>
+          <t>870135086 rev.1 (dated 2026-07-01, revize 10.07.2026)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Transit document (T1) MRN</t>
+          <t>Reference pro fakturu</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>26CH07OJWS5T87AUJ5</t>
+          <t>136782-0-0-00-FRP</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Incoterms</t>
+          <t>Freight (per shipper email)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DAP Trutnov (Incoterms 2020)</t>
+          <t>10 000 CZK — DAP Trutnov: doprava je již v ceně zboží, do celní hodnoty se nepřipočítává</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>Truck / SPZ</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CHF</t>
+          <t>AA152PU — příjezd 10.07., nejpozději 13.07.2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Country of origin</t>
+          <t>Transit document (T1) MRN</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>TW (Taiwan) — all items</t>
+          <t>26CH07OJWS5T87AUJ5</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>Incoterms</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>DAP Trutnov (Incoterms 2020)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>CHF</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Country of origin</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>TW (Taiwan) — all items</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>Packages</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>2 pallets (HU 10002844646, 10002844647)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>HS code</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Net weight (kg)</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>Gross weight (kg)</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>Customs value (CHF)</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>COO</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>CBAM</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr">
+      <c r="J17" s="3" t="inlineStr">
         <is>
           <t>Antidumping</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>8471500000</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Servery MOXA DA820E (výpočetní jednotky) – Station / REMACC / Engineering / Historian Servers [EN: MOXA DA820E CONFIGURED]</t>
         </is>
       </c>
-      <c r="C15" s="6" t="n">
+      <c r="C18" s="6" t="n">
         <v>144</v>
       </c>
-      <c r="D15" s="6" t="n">
-        <v>153</v>
-      </c>
-      <c r="E15" s="4" t="n">
+      <c r="D18" s="6" t="n">
+        <v>156.5</v>
+      </c>
+      <c r="E18" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="G18" s="7" t="n">
         <v>164538</v>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>TW</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr">
+      <c r="J18" s="4" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>8517620000</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Síťové prvky MOXA – ethernetové přepínače, moduly rozhraní a SFP transceivery [EN: RKS-G4028-4GS-2HV-T, RM-G4000-8GSFP/-8SFP/-8GTX, PT-G510-8GTX-PHR-HV, SFP-1GLSXLC-T, SFP-1FEMLC-T]</t>
         </is>
       </c>
-      <c r="C16" s="6" t="n">
+      <c r="C19" s="6" t="n">
         <v>224</v>
       </c>
-      <c r="D16" s="6" t="n">
-        <v>255</v>
-      </c>
-      <c r="E16" s="4" t="n">
+      <c r="D19" s="6" t="n">
+        <v>260.83</v>
+      </c>
+      <c r="E19" s="4" t="n">
         <v>336</v>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="G16" s="7" t="n">
+      <c r="G19" s="7" t="n">
         <v>63610</v>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>TW</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="I19" s="4" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr">
+      <c r="J19" s="4" t="inlineStr">
         <is>
           <t>Ne</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B17" s="8" t="n"/>
-      <c r="C17" s="9" t="n">
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="9" t="n">
         <v>368</v>
       </c>
-      <c r="D17" s="9" t="n">
-        <v>408</v>
-      </c>
-      <c r="E17" s="8" t="n">
+      <c r="D20" s="9" t="n">
+        <v>417.33</v>
+      </c>
+      <c r="E20" s="8" t="n">
         <v>348</v>
       </c>
-      <c r="F17" s="8" t="n"/>
-      <c r="G17" s="10" t="n">
+      <c r="F20" s="8" t="n"/>
+      <c r="G20" s="10" t="n">
         <v>228148</v>
       </c>
-      <c r="H17" s="8" t="n"/>
-      <c r="I17" s="8" t="n"/>
-      <c r="J17" s="8" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+      <c r="H20" s="8" t="n"/>
+      <c r="I20" s="8" t="n"/>
+      <c r="J20" s="8" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>⚠ PREFERENČNÍ VĚTA: NENALEZENA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>Faktura ani průvodní doklady neobsahují prohlášení o preferenčním původu. Zboží je původem z Tchaj-wanu (TW) — preferenční zacházení se neuplatní, platí standardní třetizemní sazba (u HS 8471 50 a 8517 62 je smluvní sazba EU 0 %).</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="12" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="13" t="inlineStr">
-        <is>
-          <t>Poznámky / Notes:</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="12" t="inlineStr">
         <is>
+          <t>Faktura ani průvodní doklady neobsahují prohlášení o preferenčním původu. Zboží je původem z Tchaj-wanu (TW) — preferenční zacházení se neuplatní, platí standardní třetizemní sazba (u HS 8471 50 a 8517 62 je smluvní sazba EU 0 %).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>Poznámky / Notes:</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
           <t>• Popisy: zdrojové doklady neobsahují české popisy zboží — český popis je překlad, v hranatých závorkách je originální anglický text z faktury.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="12" t="inlineStr">
-        <is>
-          <t>• Hmotnosti dle e-mailu odesílatele (M. Jahnholz, Hitachi Energy) per produktová řada: Moxa DA 12 ks NW 144 / GW 153 kg; RKS 20 ks NW 104 / GW 115 kg; RM 52 ks NW 10 / GW 15 kg; PT 4 ks NW 6 / GW 10 kg; SFP 260 ks NW 104 / GW 115 kg. Součty (NW 368 / GW 408 kg) souhlasí s fakturou i balicím listem.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>• Nesoulad s T1: tranzitní doklad deklaruje hrubou hmotnost celkem 417,33 kg (vs. 408,00 kg) a jiné rozdělení vah na pozice (HS 847150: NW 189,33 kg vs. 144 kg dle odesílatele).</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="11" t="inlineStr">
-        <is>
-          <t>• Množství dle faktury (12 ks serverů). Pozor: T1 deklaruje u HS 847150 celkem 16 ks (pozice 1,2,3,4,13 = 4+4+2+2+4), faktura, balicí list i e-mail odesílatele mají 12 ks — pravděpodobně duplicitní pozice v T1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
+    <row r="27" ht="30" customHeight="1">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>• CBAM: nevztahuje se — elektronika/IT zařízení nespadá do působnosti CBAM.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
+          <t>• REVIZE 10.07.2026 (rev.1 od M. Jahnholze): hrubá hmotnost na faktuře opravena z 408,00 na 417,33 kg (= T1) a balicí list na 160 + 257 kg za palety. Čisté hmotnosti (368,00 kg) a množství beze změny.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>• Antidumping: na uvedené HS kódy původu TW nejsou známa antidumpingová cla.</t>
+          <t>• Čisté hmotnosti per HS dle e-mailu odesílatele (Moxa DA 144 kg / síťové prvky 224 kg). Hrubá hmotnost 417,33 kg rozdělena na HS kódy proporcionálně dle původních vah produktových řad (153 : 255) → 156,50 / 260,83 kg.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="12" t="inlineStr">
-        <is>
-          <t>• Obchodní sleva: žádná sleva na faktuře — celní hodnoty = fakturované částky (celkem 228 148,00 CHF).</t>
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>• Množství: 12 ks serverů potvrzeno i v rev.1 faktury a balicího listu. Původní T1 deklaroval 16 ks (duplicitní pozice 13) — opravený T1 jsme zatím neobdrželi, nutno ověřit, že duplicitní pozice byla odstraněna.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="12" t="inlineStr">
         <is>
+          <t>• Drobnost: palety v rev.1 balicího listu = 160 + 257 = 417,00 kg vs. faktura 417,33 kg (rozdíl 0,33 kg, zaokrouhlení).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>• CBAM: nevztahuje se — elektronika/IT zařízení nespadá do působnosti CBAM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>• Antidumping: na uvedené HS kódy původu TW nejsou známa antidumpingová cla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>• Obchodní sleva: žádná sleva na faktuře — celní hodnoty = fakturované částky (celkem 228 148,00 CHF).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
           <t>• Doklad T1: zboží se švýcarským statusem T1, celní úřad určení celní úřad Hradec Králové (CZ). Lhůta pro předložení: 17.07.2026.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="A23:J23"/>
+    <mergeCell ref="A32:J32"/>
+    <mergeCell ref="A31:J31"/>
     <mergeCell ref="A22:J22"/>
     <mergeCell ref="A27:J27"/>
-    <mergeCell ref="A21:J21"/>
+    <mergeCell ref="A30:J30"/>
     <mergeCell ref="A28:J28"/>
-    <mergeCell ref="A30:J30"/>
+    <mergeCell ref="A34:J34"/>
     <mergeCell ref="A29:J29"/>
-    <mergeCell ref="A20:J20"/>
+    <mergeCell ref="A26:J26"/>
     <mergeCell ref="A24:J24"/>
-    <mergeCell ref="A26:J26"/>
     <mergeCell ref="A25:J25"/>
-    <mergeCell ref="A19:J19"/>
+    <mergeCell ref="A33:J33"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>